<commit_message>
Daily local update (bizportal/BOI blocked from GitHub)
</commit_message>
<xml_diff>
--- a/ytm_computed.xlsx
+++ b/ytm_computed.xlsx
@@ -943,22 +943,22 @@
         <v>1082</v>
       </c>
       <c r="AY2" s="11" t="n">
-        <v>0.07933805140800142</v>
+        <v>0.07936694795839348</v>
       </c>
       <c r="AZ2" s="12" t="n">
         <v>0.8396670285921102</v>
       </c>
       <c r="BA2" s="8" t="n">
-        <v>3.064566043442644</v>
+        <v>3.061811658736304</v>
       </c>
       <c r="BB2" s="8" t="n">
-        <v>2.839301402785627</v>
+        <v>2.836673537695105</v>
       </c>
       <c r="BC2" s="8" t="n">
-        <v>3.298630136986302</v>
+        <v>3.295890410958904</v>
       </c>
       <c r="BD2" s="11" t="n">
-        <v>0.003263104745742824</v>
+        <v>0.003266040212325563</v>
       </c>
       <c r="BE2" s="1" t="n"/>
       <c r="BF2" s="1" t="n"/>
@@ -1054,22 +1054,22 @@
         <v>1036</v>
       </c>
       <c r="AY3" s="11" t="n">
-        <v>-0.001419704509683132</v>
+        <v>-0.001489967301211758</v>
       </c>
       <c r="AZ3" s="12" t="n">
         <v>0.1004841921884687</v>
       </c>
       <c r="BA3" s="8" t="n">
-        <v>1.775026592299674</v>
+        <v>1.772289835737123</v>
       </c>
       <c r="BB3" s="8" t="n">
-        <v>1.777550188318217</v>
+        <v>1.774934429999617</v>
       </c>
       <c r="BC3" s="8" t="n">
-        <v>1.794520547945206</v>
+        <v>1.791780821917808</v>
       </c>
       <c r="BD3" s="11" t="n">
-        <v>0.005633718414913597</v>
+        <v>0.005642417960288558</v>
       </c>
     </row>
     <row r="4">
@@ -1163,22 +1163,22 @@
         <v>1978</v>
       </c>
       <c r="AY4" s="11" t="n">
-        <v>0.01741187511267556</v>
+        <v>0.01739731748957968</v>
       </c>
       <c r="AZ4" s="12" t="n">
         <v>0.1961473087818697</v>
       </c>
       <c r="BA4" s="8" t="n">
-        <v>4.427851447800052</v>
+        <v>4.425126424476521</v>
       </c>
       <c r="BB4" s="8" t="n">
-        <v>4.352073684327382</v>
+        <v>4.349457530903942</v>
       </c>
       <c r="BC4" s="8" t="n">
-        <v>4.794520547945205</v>
+        <v>4.791780821917809</v>
       </c>
       <c r="BD4" s="11" t="n">
-        <v>0.002258431683603214</v>
+        <v>0.002259822441385495</v>
       </c>
     </row>
     <row r="5">
@@ -1272,22 +1272,22 @@
         <v>2101</v>
       </c>
       <c r="AY5" s="11" t="n">
-        <v>0.04301304434440664</v>
+        <v>0.04327649450424095</v>
       </c>
       <c r="AZ5" s="12" t="n">
         <v>1.50729086722947</v>
       </c>
       <c r="BA5" s="8" t="n">
-        <v>0.3232876712328767</v>
+        <v>0.3205479452054794</v>
       </c>
       <c r="BB5" s="8" t="n">
-        <v>0.3099555398524105</v>
+        <v>0.3072511907380813</v>
       </c>
       <c r="BC5" s="8" t="n">
-        <v>0.2958904109589041</v>
+        <v>0.2931506849315069</v>
       </c>
       <c r="BD5" s="11" t="n">
-        <v>0.03093220338983051</v>
+        <v>0.0311965811965812</v>
       </c>
     </row>
     <row r="6">
@@ -1399,22 +1399,22 @@
         <v>720</v>
       </c>
       <c r="AY6" s="11" t="n">
-        <v>-0.1260564998452855</v>
+        <v>-0.1261102128347981</v>
       </c>
       <c r="AZ6" s="12" t="n">
         <v>0.02967633459436736</v>
       </c>
       <c r="BA6" s="8" t="n">
-        <v>6.591035006641104</v>
+        <v>6.588384367909246</v>
       </c>
       <c r="BB6" s="8" t="n">
-        <v>7.541717520039101</v>
+        <v>7.539147916216309</v>
       </c>
       <c r="BC6" s="8" t="n">
-        <v>6.96986301369863</v>
+        <v>6.967123287671233</v>
       </c>
       <c r="BD6" s="11" t="n">
-        <v>0.001517212393793089</v>
+        <v>0.001517822798667922</v>
       </c>
     </row>
     <row r="7">
@@ -1508,22 +1508,22 @@
         <v>720</v>
       </c>
       <c r="AY7" s="11" t="n">
-        <v>-0.06872717362335951</v>
+        <v>-0.06882707861034022</v>
       </c>
       <c r="AZ7" s="12" t="n">
         <v>0.1793190416141235</v>
       </c>
       <c r="BA7" s="8" t="n">
-        <v>1.984895999251951</v>
+        <v>1.982157006729311</v>
       </c>
       <c r="BB7" s="8" t="n">
-        <v>2.131379702095149</v>
+        <v>2.128666933066726</v>
       </c>
       <c r="BC7" s="8" t="n">
-        <v>1.967123287671233</v>
+        <v>1.964383561643836</v>
       </c>
       <c r="BD7" s="11" t="n">
-        <v>0.005038047335361</v>
+        <v>0.005045009031096208</v>
       </c>
     </row>
     <row r="8">
@@ -1617,22 +1617,22 @@
         <v>1581</v>
       </c>
       <c r="AY8" s="11" t="n">
-        <v>0.04139007075187335</v>
+        <v>0.04150736046731679</v>
       </c>
       <c r="AZ8" s="12" t="n">
         <v>2.787238494883721</v>
       </c>
       <c r="BA8" s="8" t="n">
-        <v>0.9068493150684933</v>
+        <v>0.904109589041096</v>
       </c>
       <c r="BB8" s="8" t="n">
-        <v>0.8708065695438763</v>
+        <v>0.8680779640726001</v>
       </c>
       <c r="BC8" s="8" t="n">
-        <v>0.8794520547945206</v>
+        <v>0.8767123287671232</v>
       </c>
       <c r="BD8" s="11" t="n">
-        <v>0.01102719033232628</v>
+        <v>0.01106060606060606</v>
       </c>
     </row>
     <row r="9">
@@ -1729,22 +1729,22 @@
         <v>1975</v>
       </c>
       <c r="AY9" s="11" t="n">
-        <v>0.1573397499420458</v>
+        <v>0.157514763817518</v>
       </c>
       <c r="AZ9" s="12" t="n">
         <v>3.191204188481676</v>
       </c>
       <c r="BA9" s="8" t="n">
-        <v>1.686457740310068</v>
+        <v>1.683711133019195</v>
       </c>
       <c r="BB9" s="8" t="n">
-        <v>1.457184668887868</v>
+        <v>1.454591496929392</v>
       </c>
       <c r="BC9" s="8" t="n">
-        <v>1.715068493150685</v>
+        <v>1.712328767123288</v>
       </c>
       <c r="BD9" s="11" t="n">
-        <v>0.005929588249369015</v>
+        <v>0.005939261078631827</v>
       </c>
     </row>
     <row r="10">
@@ -1859,22 +1859,22 @@
         <v>1884</v>
       </c>
       <c r="AY10" s="2" t="n">
-        <v>-0.008904454160736168</v>
+        <v>-0.008921797620944279</v>
       </c>
       <c r="AZ10" s="3" t="n">
         <v>0.2873038516405135</v>
       </c>
       <c r="BA10" s="4" t="n">
-        <v>4.145991754994926</v>
+        <v>4.143260758574742</v>
       </c>
       <c r="BB10" s="4" t="n">
-        <v>4.183241234813625</v>
+        <v>4.1805588586541</v>
       </c>
       <c r="BC10" s="4" t="n">
-        <v>4.304109589041096</v>
+        <v>4.301369863013699</v>
       </c>
       <c r="BD10" s="2" t="n">
-        <v>0.002411968134753862</v>
+        <v>0.002413557963810113</v>
       </c>
       <c r="BE10" s="1" t="n">
         <v>3.73</v>
@@ -1996,22 +1996,22 @@
         <v>126</v>
       </c>
       <c r="AY11" s="11" t="n">
-        <v>0.03453665253624356</v>
+        <v>0.03451781623499121</v>
       </c>
       <c r="AZ11" s="12" t="n">
         <v>0.3869382285714287</v>
       </c>
       <c r="BA11" s="8" t="n">
-        <v>2.672759854245121</v>
+        <v>2.670024269806977</v>
       </c>
       <c r="BB11" s="8" t="n">
-        <v>2.583533263604195</v>
+        <v>2.580935995403369</v>
       </c>
       <c r="BC11" s="8" t="n">
-        <v>2.794520547945206</v>
+        <v>2.791780821917808</v>
       </c>
       <c r="BD11" s="11" t="n">
-        <v>0.003741450988990683</v>
+        <v>0.003745284308117142</v>
       </c>
     </row>
     <row r="12">
@@ -2111,7 +2111,7 @@
       <c r="BA12" s="8" t="n"/>
       <c r="BB12" s="8" t="n"/>
       <c r="BC12" s="8" t="n">
-        <v>-0.03013698630136986</v>
+        <v>-0.03287671232876712</v>
       </c>
       <c r="BD12" s="11" t="n"/>
       <c r="BE12" s="1" t="n"/>
@@ -2208,22 +2208,22 @@
         <v>1006</v>
       </c>
       <c r="AY13" s="11" t="n">
-        <v>-0.1394013434770847</v>
+        <v>-0.1394967433807071</v>
       </c>
       <c r="AZ13" s="12" t="n">
         <v>0.005499153976311177</v>
       </c>
       <c r="BA13" s="8" t="n">
-        <v>4.279091147352849</v>
+        <v>4.276434385703712</v>
       </c>
       <c r="BB13" s="8" t="n">
-        <v>4.97222615317772</v>
+        <v>4.969689949233635</v>
       </c>
       <c r="BC13" s="8" t="n">
-        <v>4.545205479452055</v>
+        <v>4.542465753424658</v>
       </c>
       <c r="BD13" s="11" t="n">
-        <v>0.002336944845446035</v>
+        <v>0.002338396687069581</v>
       </c>
     </row>
     <row r="14">
@@ -2317,22 +2317,22 @@
         <v>1769</v>
       </c>
       <c r="AY14" s="11" t="n">
-        <v>-0.2031704219051334</v>
+        <v>-0.2033372284000346</v>
       </c>
       <c r="AZ14" s="12" t="n">
         <v>-0.02357024641412286</v>
       </c>
       <c r="BA14" s="8" t="n">
-        <v>3.19498382071986</v>
+        <v>3.192299761392695</v>
       </c>
       <c r="BB14" s="8" t="n">
-        <v>4.00962000978769</v>
+        <v>4.007090421686818</v>
       </c>
       <c r="BC14" s="8" t="n">
-        <v>3.298630136986302</v>
+        <v>3.295890410958904</v>
       </c>
       <c r="BD14" s="11" t="n">
-        <v>0.003129906303483848</v>
+        <v>0.003132537902905876</v>
       </c>
     </row>
     <row r="15">
@@ -2426,22 +2426,22 @@
         <v>1532</v>
       </c>
       <c r="AY15" s="11" t="n">
-        <v>-0.1676665548859828</v>
+        <v>-0.1679301089997484</v>
       </c>
       <c r="AZ15" s="12" t="n">
         <v>0.1359308176100629</v>
       </c>
       <c r="BA15" s="8" t="n">
-        <v>1.942040282390118</v>
+        <v>1.939362913427614</v>
       </c>
       <c r="BB15" s="8" t="n">
-        <v>2.333247923401765</v>
+        <v>2.330769247155739</v>
       </c>
       <c r="BC15" s="8" t="n">
-        <v>2.06027397260274</v>
+        <v>2.057534246575342</v>
       </c>
       <c r="BD15" s="11" t="n">
-        <v>0.005149223778042724</v>
+        <v>0.005156332489789693</v>
       </c>
     </row>
     <row r="16">
@@ -2535,22 +2535,22 @@
         <v>767</v>
       </c>
       <c r="AY16" s="11" t="n">
-        <v>-0.04313280495115236</v>
+        <v>-0.04322939202460834</v>
       </c>
       <c r="AZ16" s="12" t="n">
         <v>0.11487679160105</v>
       </c>
       <c r="BA16" s="8" t="n">
-        <v>1.796372108842995</v>
+        <v>1.793634632376511</v>
       </c>
       <c r="BB16" s="8" t="n">
-        <v>1.87734736663356</v>
+        <v>1.874675724175929</v>
       </c>
       <c r="BC16" s="8" t="n">
-        <v>1.794520547945206</v>
+        <v>1.791780821917808</v>
       </c>
       <c r="BD16" s="11" t="n">
-        <v>0.00556677536395329</v>
+        <v>0.005575271473627996</v>
       </c>
     </row>
     <row r="17">
@@ -2665,22 +2665,22 @@
         <v>486</v>
       </c>
       <c r="AY17" s="11" t="n">
-        <v>0.0594240010861711</v>
+        <v>0.05943166088291226</v>
       </c>
       <c r="AZ17" s="12" t="n">
         <v>0.876214196762142</v>
       </c>
       <c r="BA17" s="8" t="n">
-        <v>3.041336045730312</v>
+        <v>3.038592073359466</v>
       </c>
       <c r="BB17" s="8" t="n">
-        <v>2.870744897805027</v>
+        <v>2.868134100152487</v>
       </c>
       <c r="BC17" s="8" t="n">
-        <v>3.298630136986302</v>
+        <v>3.295890410958904</v>
       </c>
       <c r="BD17" s="11" t="n">
-        <v>0.003288028632692154</v>
+        <v>0.003290997856432898</v>
       </c>
     </row>
     <row r="18">
@@ -2795,22 +2795,22 @@
         <v>2386</v>
       </c>
       <c r="AY18" s="11" t="n">
-        <v>0.1342600958392862</v>
+        <v>0.1343818729218592</v>
       </c>
       <c r="AZ18" s="12" t="n">
         <v>1.723901712583767</v>
       </c>
       <c r="BA18" s="8" t="n">
-        <v>1.767933536816058</v>
+        <v>1.76518859100561</v>
       </c>
       <c r="BB18" s="8" t="n">
-        <v>1.558666784894597</v>
+        <v>1.556079688102706</v>
       </c>
       <c r="BC18" s="8" t="n">
-        <v>1.794520547945206</v>
+        <v>1.791780821917808</v>
       </c>
       <c r="BD18" s="11" t="n">
-        <v>0.005656321231401831</v>
+        <v>0.005665117059420321</v>
       </c>
     </row>
     <row r="19">
@@ -2904,22 +2904,22 @@
         <v>1238</v>
       </c>
       <c r="AY19" s="11" t="n">
-        <v>0.02997720850254504</v>
+        <v>0.02996463335001393</v>
       </c>
       <c r="AZ19" s="12" t="n">
         <v>0.3969162995594715</v>
       </c>
       <c r="BA19" s="8" t="n">
-        <v>3.230151943254585</v>
+        <v>3.227418733510775</v>
       </c>
       <c r="BB19" s="8" t="n">
-        <v>3.136139243266181</v>
+        <v>3.133523840535598</v>
       </c>
       <c r="BC19" s="8" t="n">
-        <v>3.46027397260274</v>
+        <v>3.457534246575342</v>
       </c>
       <c r="BD19" s="11" t="n">
-        <v>0.003095829600487573</v>
+        <v>0.003098451371112305</v>
       </c>
     </row>
     <row r="20">
@@ -3013,22 +3013,22 @@
         <v>224</v>
       </c>
       <c r="AY20" s="11" t="n">
-        <v>-0.5534178248595648</v>
+        <v>-0.554094953443287</v>
       </c>
       <c r="AZ20" s="12" t="n">
         <v>-0.005458803178042593</v>
       </c>
       <c r="BA20" s="8" t="n">
-        <v>1.472913967956809</v>
+        <v>1.470192244828508</v>
       </c>
       <c r="BB20" s="8" t="n">
-        <v>3.298192471505669</v>
+        <v>3.29709712007379</v>
       </c>
       <c r="BC20" s="8" t="n">
-        <v>1.457534246575342</v>
+        <v>1.454794520547945</v>
       </c>
       <c r="BD20" s="11" t="n">
-        <v>0.006789262793041306</v>
+        <v>0.006801831553101725</v>
       </c>
       <c r="BE20" s="1" t="n"/>
       <c r="BF20" s="1" t="n"/>
@@ -3124,22 +3124,22 @@
         <v>473</v>
       </c>
       <c r="AY21" s="11" t="n">
-        <v>0.03081254519161238</v>
+        <v>0.03079343055587937</v>
       </c>
       <c r="AZ21" s="12" t="n">
         <v>0.3329002449624654</v>
       </c>
       <c r="BA21" s="8" t="n">
-        <v>0.8219178082191779</v>
+        <v>0.8191780821917809</v>
       </c>
       <c r="BB21" s="8" t="n">
-        <v>0.7973494424889793</v>
+        <v>0.7947063474686873</v>
       </c>
       <c r="BC21" s="8" t="n">
-        <v>0.7945205479452054</v>
+        <v>0.7917808219178082</v>
       </c>
       <c r="BD21" s="11" t="n">
-        <v>0.01216666666666667</v>
+        <v>0.01220735785953177</v>
       </c>
       <c r="BE21" s="1" t="n"/>
       <c r="BF21" s="1" t="n"/>
@@ -3259,22 +3259,22 @@
         <v>345</v>
       </c>
       <c r="AY22" s="11" t="n">
-        <v>0.08854561954375785</v>
+        <v>0.08857257752479575</v>
       </c>
       <c r="AZ22" s="12" t="n">
         <v>0.09718518518518504</v>
       </c>
       <c r="BA22" s="8" t="n">
-        <v>1.877015427525002</v>
+        <v>1.874268442071271</v>
       </c>
       <c r="BB22" s="8" t="n">
-        <v>1.724333269846527</v>
+        <v>1.721767092767481</v>
       </c>
       <c r="BC22" s="8" t="n">
-        <v>2.06027397260274</v>
+        <v>2.057534246575342</v>
       </c>
       <c r="BD22" s="11" t="n">
-        <v>0.00532760671721586</v>
+        <v>0.005335415021419723</v>
       </c>
     </row>
     <row r="23">
@@ -3368,22 +3368,22 @@
         <v>445</v>
       </c>
       <c r="AY23" s="11" t="n">
-        <v>0.02030341822375703</v>
+        <v>0.02031289274274506</v>
       </c>
       <c r="AZ23" s="12" t="n">
         <v>0.4923064752941175</v>
       </c>
       <c r="BA23" s="8" t="n">
-        <v>4.361928076590014</v>
+        <v>4.359186923610526</v>
       </c>
       <c r="BB23" s="8" t="n">
-        <v>4.275128357585707</v>
+        <v>4.272402078437347</v>
       </c>
       <c r="BC23" s="8" t="n">
-        <v>4.386301369863014</v>
+        <v>4.383561643835616</v>
       </c>
       <c r="BD23" s="11" t="n">
-        <v>0.002292564165298574</v>
+        <v>0.002294005780260836</v>
       </c>
     </row>
     <row r="24" customFormat="1" s="1">
@@ -3477,22 +3477,22 @@
         <v>544</v>
       </c>
       <c r="AY24" s="11" t="n">
-        <v>0.1731658307852075</v>
+        <v>0.1732606661931288</v>
       </c>
       <c r="AZ24" s="12" t="n">
         <v>0.4108097665653494</v>
       </c>
       <c r="BA24" s="8" t="n">
-        <v>2.947644383250005</v>
+        <v>2.944842619433716</v>
       </c>
       <c r="BB24" s="8" t="n">
-        <v>2.51255560458757</v>
+        <v>2.509964498331668</v>
       </c>
       <c r="BC24" s="8" t="n">
-        <v>3.298630136986302</v>
+        <v>3.295890410958904</v>
       </c>
       <c r="BD24" s="11" t="n">
-        <v>0.003392539499277802</v>
+        <v>0.003395767208070009</v>
       </c>
     </row>
     <row r="25" customFormat="1" s="1">
@@ -3586,22 +3586,22 @@
         <v>494</v>
       </c>
       <c r="AY25" s="11" t="n">
-        <v>0.2416653757838158</v>
+        <v>0.2418240169266165</v>
       </c>
       <c r="AZ25" s="12" t="n">
         <v>0.9283387622149839</v>
       </c>
       <c r="BA25" s="8" t="n">
-        <v>2.931498734885361</v>
+        <v>2.9286561213125</v>
       </c>
       <c r="BB25" s="8" t="n">
-        <v>2.360941032953277</v>
+        <v>2.358350363170311</v>
       </c>
       <c r="BC25" s="8" t="n">
-        <v>3.298630136986302</v>
+        <v>3.295890410958904</v>
       </c>
       <c r="BD25" s="11" t="n">
-        <v>0.003411224395561971</v>
+        <v>0.003414535399778661</v>
       </c>
       <c r="BF25" s="16" t="n"/>
     </row>
@@ -3699,22 +3699,22 @@
         <v>1502</v>
       </c>
       <c r="AY26" s="11" t="n">
-        <v>63.70910408785361</v>
+        <v>64.21418062811505</v>
       </c>
       <c r="AZ26" s="12" t="n">
         <v>-0.02843478260869559</v>
       </c>
       <c r="BA26" s="8" t="n">
-        <v>0.3232876712328767</v>
+        <v>0.3205479452054794</v>
       </c>
       <c r="BB26" s="8" t="n">
-        <v>0.004996015256121592</v>
+        <v>0.004915310475698674</v>
       </c>
       <c r="BC26" s="8" t="n">
-        <v>0.2958904109589041</v>
+        <v>0.2931506849315069</v>
       </c>
       <c r="BD26" s="11" t="n">
-        <v>0.03093220338983051</v>
+        <v>0.0311965811965812</v>
       </c>
     </row>
     <row r="27">
@@ -3808,22 +3808,22 @@
         <v>1484</v>
       </c>
       <c r="AY27" s="11" t="n">
-        <v>0.0552794232017451</v>
+        <v>0.05551915230425707</v>
       </c>
       <c r="AZ27" s="12" t="n">
         <v>0.4600450863024543</v>
       </c>
       <c r="BA27" s="8" t="n">
-        <v>0.3178082191780822</v>
+        <v>0.3150684931506849</v>
       </c>
       <c r="BB27" s="8" t="n">
-        <v>0.3011602540432788</v>
+        <v>0.2984962352060338</v>
       </c>
       <c r="BC27" s="8" t="n">
-        <v>0.2958904109589041</v>
+        <v>0.2931506849315069</v>
       </c>
       <c r="BD27" s="11" t="n">
-        <v>0.03146551724137931</v>
+        <v>0.03173913043478261</v>
       </c>
     </row>
     <row r="28" customFormat="1" s="1">
@@ -3938,7 +3938,7 @@
         <v>1688</v>
       </c>
       <c r="AY28" s="11" t="n">
-        <v>-2.472428403982761</v>
+        <v>-2.493576663511783</v>
       </c>
       <c r="AZ28" s="12" t="n">
         <v>0.0429346862835247</v>
@@ -3946,7 +3946,7 @@
       <c r="BA28" s="8" t="n"/>
       <c r="BB28" s="8" t="n"/>
       <c r="BC28" s="8" t="n">
-        <v>0.2958904109589041</v>
+        <v>0.2931506849315069</v>
       </c>
       <c r="BD28" s="11" t="n"/>
     </row>
@@ -4059,22 +4059,22 @@
         <v>1831</v>
       </c>
       <c r="AY29" s="11" t="n">
-        <v>-0.1734919144781247</v>
+        <v>-0.173672007819939</v>
       </c>
       <c r="AZ29" s="12" t="n">
         <v>0.1997923913043478</v>
       </c>
       <c r="BA29" s="8" t="n">
-        <v>2.724504393160848</v>
+        <v>2.721797048763548</v>
       </c>
       <c r="BB29" s="8" t="n">
-        <v>3.296403799172196</v>
+        <v>3.293845875392365</v>
       </c>
       <c r="BC29" s="8" t="n">
-        <v>2.794520547945206</v>
+        <v>2.791780821917808</v>
       </c>
       <c r="BD29" s="11" t="n">
-        <v>0.003670392319829754</v>
+        <v>0.003674043222488899</v>
       </c>
     </row>
     <row r="30">
@@ -4189,22 +4189,22 @@
         <v>1974</v>
       </c>
       <c r="AY30" s="11" t="n">
-        <v>0.05374397913901684</v>
+        <v>0.05374186556903203</v>
       </c>
       <c r="AZ30" s="12" t="n">
         <v>0.5663390856685349</v>
       </c>
       <c r="BA30" s="8" t="n">
-        <v>2.668516414273173</v>
+        <v>2.665777157407037</v>
       </c>
       <c r="BB30" s="8" t="n">
-        <v>2.532414388221264</v>
+        <v>2.529819915589562</v>
       </c>
       <c r="BC30" s="8" t="n">
-        <v>2.794520547945206</v>
+        <v>2.791780821917808</v>
       </c>
       <c r="BD30" s="11" t="n">
-        <v>0.003747400595519181</v>
+        <v>0.003751251289784048</v>
       </c>
       <c r="BE30" s="1" t="n"/>
       <c r="BF30" s="1" t="n"/>
@@ -4303,22 +4303,22 @@
         <v>1369</v>
       </c>
       <c r="AY31" s="11" t="n">
-        <v>0.1162872076857349</v>
+        <v>0.1163455898826516</v>
       </c>
       <c r="AZ31" s="12" t="n">
         <v>0.9999969127710844</v>
       </c>
       <c r="BA31" s="8" t="n">
-        <v>2.203140899177193</v>
+        <v>2.200386354254198</v>
       </c>
       <c r="BB31" s="8" t="n">
-        <v>1.973632667299576</v>
+        <v>1.971061984923055</v>
       </c>
       <c r="BC31" s="8" t="n">
-        <v>2.367123287671233</v>
+        <v>2.364383561643836</v>
       </c>
       <c r="BD31" s="11" t="n">
-        <v>0.004538974336019409</v>
+        <v>0.004544656433024197</v>
       </c>
     </row>
     <row r="32">
@@ -4412,22 +4412,22 @@
         <v>1621</v>
       </c>
       <c r="AY32" s="11" t="n">
-        <v>-0.269177550711442</v>
+        <v>-0.2695814621855814</v>
       </c>
       <c r="AZ32" s="12" t="n">
         <v>0.0355780770769436</v>
       </c>
       <c r="BA32" s="8" t="n">
-        <v>1.66581061895804</v>
+        <v>1.663085590362606</v>
       </c>
       <c r="BB32" s="8" t="n">
-        <v>2.279364325192358</v>
+        <v>2.276894005646329</v>
       </c>
       <c r="BC32" s="8" t="n">
-        <v>1.668493150684931</v>
+        <v>1.665753424657534</v>
       </c>
       <c r="BD32" s="11" t="n">
-        <v>0.006003083355450676</v>
+        <v>0.00601291963441261</v>
       </c>
     </row>
     <row r="33">
@@ -4521,22 +4521,22 @@
         <v>1949</v>
       </c>
       <c r="AY33" s="11" t="n">
-        <v>-0.1016938701876407</v>
+        <v>-0.1018239118184073</v>
       </c>
       <c r="AZ33" s="12" t="n">
         <v>-0.004308472121650975</v>
       </c>
       <c r="BA33" s="8" t="n">
-        <v>2.701641821806364</v>
+        <v>2.698928597655358</v>
       </c>
       <c r="BB33" s="8" t="n">
-        <v>3.007484566949009</v>
+        <v>3.00489918755184</v>
       </c>
       <c r="BC33" s="8" t="n">
-        <v>2.794520547945206</v>
+        <v>2.791780821917808</v>
       </c>
       <c r="BD33" s="11" t="n">
-        <v>0.003701452916254394</v>
+        <v>0.003705173974845911</v>
       </c>
     </row>
     <row r="34">
@@ -4630,22 +4630,22 @@
         <v>634</v>
       </c>
       <c r="AY34" s="11" t="n">
-        <v>0.02996162326981591</v>
+        <v>0.02993850585125143</v>
       </c>
       <c r="AZ34" s="12" t="n">
         <v>0.2283621837549934</v>
       </c>
       <c r="BA34" s="8" t="n">
-        <v>1.697257207688833</v>
+        <v>1.694518394390382</v>
       </c>
       <c r="BB34" s="8" t="n">
-        <v>1.647883930180385</v>
+        <v>1.645261716853523</v>
       </c>
       <c r="BC34" s="8" t="n">
-        <v>1.715068493150685</v>
+        <v>1.712328767123288</v>
       </c>
       <c r="BD34" s="11" t="n">
-        <v>0.005891858909008298</v>
+        <v>0.005901381792670117</v>
       </c>
     </row>
     <row r="35">

</xml_diff>